<commit_message>
Remover acentos de README.md e arquivos Python
</commit_message>
<xml_diff>
--- a/outputs/tables/parametros_revisao.xlsx
+++ b/outputs/tables/parametros_revisao.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,7 +424,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Informação</t>
+          <t>InformaÃ§Ã£o</t>
         </is>
       </c>
     </row>
@@ -455,7 +455,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Descritores</t>
+          <t>EstratÃ©gia de busca</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -463,20 +463,40 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Tipo de revisão</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
+          <t>MÃ¡ximo de artigos por base</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Data de execução</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2026-05-12 21:14:31</t>
+          <t>Tipo de revisÃ£o</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Similaridade mÃ­nima</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Data de execuÃ§Ã£o</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-05-13 08:49:51</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Backup final antes da limpeza local
</commit_message>
<xml_diff>
--- a/outputs/tables/parametros_revisao.xlsx
+++ b/outputs/tables/parametros_revisao.xlsx
@@ -424,7 +424,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>InformaÃ§Ã£o</t>
+          <t>InformaAAo</t>
         </is>
       </c>
     </row>
@@ -434,7 +434,11 @@
           <t>Tema</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>cardiomiopatia de Takotsubo</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -442,7 +446,11 @@
           <t>Ano inicial</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -450,53 +458,71 @@
           <t>Ano final</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>EstratÃ©gia de busca</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
+          <t>EstratAgia de busca</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>("Takotsubo cardiomyopathy"[Title/Abstract] OR "Takotsubo syndrome"[Title/Abstract] OR "stress cardiomyopathy"[Title/Abstract] OR "stress-induced cardiomyopathy"[Title/Abstract] OR "broken heart syndrome"[Title/Abstract] OR "apical ballooning syndrome"[Title/Abstract])
+AND
+("depression"[Title/Abstract] OR "depressive symptoms"[Title/Abstract] OR "major depression"[Title/Abstract])
+AND
+("Brazil"[Title/Abstract] OR "Brasil"[Title/Abstract] OR "Brazilian"[Title/Abstract])
+AND
+("COVID-19"[Title/Abstract] OR "SARS-CoV-2"[Title/Abstract] OR "coronavirus"[Title/Abstract])</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MÃ¡ximo de artigos por base</t>
+          <t>MAximo de artigos por base</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Tipo de revisÃ£o</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
+          <t>Tipo de revisAo</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>prisma</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Similaridade mÃ­nima</t>
+          <t>Similaridade mAnima</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Data de execuÃ§Ã£o</t>
+          <t>Data de execuAAo</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-05-13 08:49:51</t>
+          <t>2026-05-13 08:59:56</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(prisma): scientific export and maintenance sidebar
</commit_message>
<xml_diff>
--- a/outputs/tables/parametros_revisao.xlsx
+++ b/outputs/tables/parametros_revisao.xlsx
@@ -424,7 +424,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>InformaÃ§Ã£o</t>
+          <t>InformaAAo</t>
         </is>
       </c>
     </row>
@@ -434,7 +434,11 @@
           <t>Tema</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>dengue</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -442,7 +446,9 @@
           <t>Ano inicial</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
+      <c r="B3" t="n">
+        <v>2014</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -450,53 +456,73 @@
           <t>Ano final</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
+      <c r="B4" t="n">
+        <v>2026</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>EstratÃ©gia de busca</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
+          <t>EstratAgia de busca</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>(
+"dengue"[Title/Abstract]
+)
+AND
+(
+"systematic review"[Title/Abstract] OR "meta-analysis"[Title/Abstract] OR review[Publication Type]
+)
+NOT
+(
+animals[Mesh] NOT humans[Mesh]
+)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MÃ¡ximo de artigos por base</t>
+          <t>MAximo de artigos por base</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Tipo de revisÃ£o</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
+          <t>Tipo de revisAo</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Revisão sistemática</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Similaridade mÃ­nima</t>
+          <t>Similaridade mAnima</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.3</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Data de execuÃ§Ã£o</t>
+          <t>Data de execuAAo</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-05-13 08:49:51</t>
+          <t>30/06/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v1.1.0: PubMed pagination, export manager, safe filenames, citation panel and UI improvements
</commit_message>
<xml_diff>
--- a/outputs/tables/parametros_revisao.xlsx
+++ b/outputs/tables/parametros_revisao.xlsx
@@ -436,7 +436,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>dengue</t>
+          <t>Clinical studies evaluating the safety, efficacy, and use of dermocosmetic products in children, including moisturizers, cleansers, sunscreens, and topical skincare formulations for healthy skin or pediatric dermatological conditions</t>
         </is>
       </c>
     </row>
@@ -447,7 +447,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2014</v>
+        <v>2016</v>
       </c>
     </row>
     <row r="4">
@@ -469,14 +469,31 @@
       <c r="B5" t="inlineStr">
         <is>
           <t>(
-"dengue"[Title/Abstract]
+child*[Title/Abstract] OR children[Title/Abstract] OR pediatric*[Title/Abstract] OR paediatric*[Title/Abstract]
+OR infant*[Title/Abstract] OR newborn*[Title/Abstract] OR adolescent*[Title/Abstract]
+OR "Child"[Mesh] OR "Infant"[Mesh] OR "Adolescent"[Mesh] OR "Pediatrics"[Mesh]
 )
 AND
 (
-"systematic review"[Title/Abstract] OR "meta-analysis"[Title/Abstract] OR review[Publication Type]
+dermocosmetic*[Title/Abstract] OR dermo-cosmetic*[Title/Abstract] OR cosmeceutical*[Title/Abstract]
+OR cosmetic*[Title/Abstract] OR "skin care"[Title/Abstract] OR "skin care product*"[Title/Abstract]
+OR moisturizer*[Title/Abstract] OR moisturiser*[Title/Abstract] OR emollient*[Title/Abstract]
+OR sunscreen*[Title/Abstract] OR "topical product*"[Title/Abstract]
+OR "Cosmetics"[Mesh] OR "Skin Care"[Mesh] OR "Sunscreening Agents"[Mesh] OR "Emollients"[Mesh]
 )
-NOT
+AND
 (
+adverse[Title/Abstract] OR harmful[Title/Abstract] OR toxicity[Title/Abstract] OR toxic*[Title/Abstract]
+OR irritation[Title/Abstract] OR dermatitis[Title/Abstract] OR allergy[Title/Abstract] OR allergic[Title/Abstract]
+OR hypersensitivity[Title/Abstract] OR "skin reaction*"[Title/Abstract] OR "adverse effect*"[Title/Abstract]
+OR "Adverse Drug Reaction Reporting Systems"[Mesh] OR "Dermatitis"[Mesh] OR "Hypersensitivity"[Mesh]
+)
+AND
+(
+review[Title/Abstract] OR "observational study"[Title/Abstract]
+OR cohort[Title/Abstract] OR "cross-sectional"[Title/Abstract]
+)
+NOT (
 animals[Mesh] NOT humans[Mesh]
 )</t>
         </is>
@@ -489,7 +506,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>30</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="7">
@@ -500,7 +517,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Revisão sistemática</t>
+          <t>Revisão de escopo</t>
         </is>
       </c>
     </row>
@@ -511,7 +528,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.35</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="9">
@@ -522,7 +539,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>30/06/2026</t>
+          <t>02/07/2026</t>
         </is>
       </c>
     </row>

</xml_diff>